<commit_message>
Finisih scrape qld (Devon)
</commit_message>
<xml_diff>
--- a/src/scrapers/output_scrape/qld/requirements_qld.xlsx
+++ b/src/scrapers/output_scrape/qld/requirements_qld.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,6 +528,193 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Building_and_Construction_Workforce_Pathway</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Occupation
+- Have an occupation on the Queensland Onshore Skills List that is indicated as included in the building and construction workforce pathway.
+Points
+- Have a score of 65 or higher in the Australian Department of Home Affairs’ points test.
+- Have a score of 65 or higher in the Australian Department of Home Affairs’ points test.
+English
+- Have at least competent English , according to the Australian Department of Home Affairs definition.
+Work experience
+- Immediately before registering your interest in Queensland nomination, you have been living and working in Queensland for the past 3 months.
+- This work experience must be:
+- After you completed your qualification
+- In an occupation that has the same first 3 digits in the Australian and New Zealand Standard Classification of Occupations (ANZSCO) code as your nominated occupation
+- At least 20 hours per week.
+- We also note the following:
+- You must still be in a role that meets the above requirements when you submit your ROI, when you are selected for invitation, and when you are nominated
+- Casual work is accepted
+- Multiple eligible jobs can be combined to meet requirements
+- Work from home is allowed, where your employer has a physical presence in Queensland.
+Visa subclass
+- Invited candidates will be nominated for the Skilled Nominated (Permanent) visa (subclass 190) unless they do not meet the Australian Department of Home Affairs’ requirements for this visa. (See our notes on 'Are you eligible for consideration' above this table.)
+- If you have applied for, or are a current holder of, a Skilled Work Regional (Provisional) visa (subclass 491), you are not eligible for nomination for the Skilled Nominated (Permanent) visa (subclass 190). This restriction also applies to the Skilled Regional (Provisional) visa (subclass 489).
+Commitment to living in Queensland
+- Commit to continue to living and working in:
+- Regional Queensland until at least 3 years after the date your Skilled Work Regional (Provisional) visa (subclass 491) is granted, or;
+- Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Graduates_of_a_Queensland_University</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Occupation
+- Have an occupation on the Queensland Onshore Skills List .
+Points
+- Have a score of 65 or higher in the Australian Department of Home Affairs’ points test.
+English
+- Have at least competent English , according to the Australian Department of Home Affairs definition.
+Study
+- You have:
+- A Bachelor Degree, Master’s Degree or PhD from a Queensland university or tertiary institute that meets the Australian Study Requirement
+- Completed 100% of this qualification in Queensland
+- Graduated after 1 July 2021.
+- Your Queensland degree does not have to be related to your nominated occupation.
+Work experience
+- Immediately before registering your interest in Queensland nomination, you have been living and working in:
+- Regional Queensland for the past 6 months for the Skilled Work Regional (Provisional) visa (subclass 491), or;
+- Queensland for the past 9 months for the Skilled Nominated (Permanent) visa (subclass 190).
+- This work experience must be:
+- After you completed your qualification
+- At least 20 hours per week.
+- Candidates who meet the Queensland university graduate requirements may be working in their nominated occupation or any Skill Level 1 occupation.
+- We also note the following:
+- You must still be in a role that meets the above requirements when you submit your ROI, when you are selected for invitation, and when you are nominated
+- Casual work is accepted
+- Multiple eligible jobs can be combined to meet requirements
+- Work from home is allowed, where your employer has a physical presence in Queensland.
+Visa subclass
+- The Queensland Onshore Skills List outlines which visa subclasses you may be nominated for based on your occupation.
+- Some occupations are only eligible for nomination for the Skilled Work Regional (Provisional) visa (subclass 491).
+- If you have applied for, or are a current holder of, a Skilled Work Regional (Provisional) visa (subclass 491), you are not eligible for nomination for the Skilled Nominated (Permanent) visa (subclass 190). This restriction also applies to the Skilled Regional (Provisional) visa (subclass 489).
+Commitment to living in Queensland
+- Commit to continue living and working in:
+- Regional Queensland until at least 3 years after the date your Skilled Work Regional (Provisional) visa (subclass 491) is granted, or;
+- Queensland until at least 2 years after the date your Skilled Nominated (Permanent) visa (subclass 190) is granted.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Small_Business_Owners</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Occupation
+- Have an occupation on the Legislative Instrument 19/051 ( LIN19/051 ) .
+Living in regional Queensland
+- Have evidence that you are living in regional Queensland in an eligible postcode.
+Location of business
+- Own and operate your business in an eligible postcode in regional Queensland.
+Ownership interest
+- Have evidence you own 100% of the business. 100% ownership is required since the business was purchased or started.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Additional requirements for Pathway 1 - Business purchase</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Time since purchase
+- Settlement of business purchase must have occurred less than 18 months before submitting your 491 SBO Registration of Interest.
+- Businesses settled before 1 July 2024 have until 31 December 2025 to submit your 491 SBO Registration of Interest.
+Age and location of purchased business
+- The business must have been operating for a minimum of 2 years in its current location, immediately before purchase, and continue to operate in the same location.
+Price of purchased business
+- Have evidence you purchased your business for a minimum of $100,000.
+Operation of business
+- Have evidence you have been operating the business for a minimum of 6 months after settlement. The 6 months of operation does not start until 100% of the business purchase price is settled.
+- You are required to submit 2 quarterly Business Activity Statements (BAS), where you have owned and operated the business for the entire period of the BAS.
+Australian employee/s
+- Have evidence of employing at least 1 Australian resident working a minimum of 20 hours per week, or 2 Australian residents working 10 hours each per week. Employees cannot be a family member or a subcontractor.
+- An Australian resident for the purposes of the 491 SBO stream is an Australian citizen, an Australian permanent resident or a New Zealand citizen residing in Australia on a Special Category visa (subclass 444).</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QLD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Additional requirements for Pathway 2 - Start up business</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Requirement
+Operation of business and turnover
+- Have evidence of operating a profitable start-up for a minimum of 2 years, with a turnover of $200,000 in the 12 months prior to submitting your 491 SBO Registration of Interest.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>